<commit_message>
Add progress UI and trim GL input rows
</commit_message>
<xml_diff>
--- a/samples/Expected_Result_Sample.xlsx
+++ b/samples/Expected_Result_Sample.xlsx
@@ -407,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -579,71 +579,10 @@
           <t>ERP bank receipt B-090</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
+      <c r="G7" s="6">
+        <f>IF(C7&gt;0,"Debit",IF(D7&gt;0,"Credit","Check"))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>